<commit_message>
Rapor: identitas siswa dari impor Excel + menu cetak per bagian
- Template impor siswa kini memuat 23 kolom identitas (agama, status
  keluarga, anak ke, asal sekolah, nama+pekerjaan ayah/ibu, alamat ortu,
  nama+pekerjaan wali) sehingga sekali impor identitas rapor terisi.
- Hapus field tinggi badan, berat badan, dan kondisi kesehatan dari form
  pelengkap rapor (UI + validasi server + test).
- Menu cetak dipecah: cover, identitas, nilai, lengkap lewat
  /api/rapor/export/pdf?bagian=...; bagian tak dikenal ditolak 400.
- Perbaiki migrasi UNIQUE per-tenant: tabel siswa/gtk/mapel dibangun ulang
  dari PRAGMA table_info, bukan daftar kolom hardcoded, sehingga kolom
  biodata tidak terhapus di DB baru (impor gagal "no column named agama").
  Recreate kini atomik (satu transaksi) dan DEFAULT ekspresi dikurung.
- Tambah e2e impor & cetak, test template impor, test runtime migrasi.
</commit_message>
<xml_diff>
--- a/public/templates/template-import-siswa.xlsx
+++ b/public/templates/template-import-siswa.xlsx
@@ -6,9 +6,6 @@
     <sheet name="Data Siswa" sheetId="1" r:id="rId1"/>
     <sheet name="Petunjuk" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Data Siswa'!A1:L2</definedName>
-  </definedNames>
 </workbook>
 </file>
 
@@ -401,20 +398,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:W2"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="13.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
     <col min="8" max="8" width="17.83203125" customWidth="1"/>
-    <col min="9" max="9" width="32.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="26.83203125" customWidth="1"/>
-    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="19.83203125" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="14" max="14" width="16.83203125" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="16.83203125" customWidth="1"/>
+    <col min="17" max="17" width="18.83203125" customWidth="1"/>
+    <col min="18" max="18" width="16.83203125" customWidth="1"/>
+    <col min="19" max="19" width="17.83203125" customWidth="1"/>
+    <col min="20" max="20" width="16.83203125" customWidth="1"/>
+    <col min="21" max="21" width="16.83203125" customWidth="1"/>
+    <col min="22" max="22" width="18.83203125" customWidth="1"/>
+    <col min="23" max="23" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,9 +457,42 @@
         <v>No HP</v>
       </c>
       <c r="K1" t="str">
+        <v>Agama</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Status Keluarga</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Anak Ke</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Asal Sekolah</v>
+      </c>
+      <c r="O1" t="str">
         <v>Nama Ortu</v>
       </c>
-      <c r="L1" t="str">
+      <c r="P1" t="str">
+        <v>Nama Ayah</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Pekerjaan Ayah</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Nama Ibu</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Pekerjaan Ibu</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Alamat Ortu</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Nama Wali</v>
+      </c>
+      <c r="V1" t="str">
+        <v>Pekerjaan Wali</v>
+      </c>
+      <c r="W1" t="str">
         <v>Rombel</v>
       </c>
     </row>
@@ -487,26 +528,58 @@
         <v>081234567890</v>
       </c>
       <c r="K2" t="str">
+        <v>Islam</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Anak Kandung</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2" t="str">
+        <v>SDN 1 Contoh</v>
+      </c>
+      <c r="O2" t="str">
         <v>Bapak/Ibu Ahmad</v>
       </c>
-      <c r="L2" t="str">
-        <v>1A</v>
+      <c r="P2" t="str">
+        <v>Slamet Riyadi</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Petani</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Siti Aminah</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Ibu Rumah Tangga</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Jl. Contoh No. 1</v>
+      </c>
+      <c r="U2" t="str">
+        <v>Kakek Ahmad</v>
+      </c>
+      <c r="V2" t="str">
+        <v>Pensiunan</v>
+      </c>
+      <c r="W2" t="str">
+        <v>7A</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L2"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B12"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+    <col min="1" max="1" width="26.83203125" customWidth="1"/>
+    <col min="2" max="2" width="74.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -514,49 +587,89 @@
         <v>PETUNJUK PENGISIAN</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Kolom wajib</v>
-      </c>
-      <c r="B2" t="str">
-        <v>NIS, Nama, dan JK. NIK jika diisi harus tepat 16 digit angka.</v>
-      </c>
-    </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>JK</v>
+        <v>Kolom wajib</v>
       </c>
       <c r="B3" t="str">
-        <v>Isi L untuk laki-laki atau P untuk perempuan.</v>
+        <v>NIS, Nama, dan JK. NIK jika diisi harus tepat 16 digit angka.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Tanggal Lahir</v>
+        <v>JK</v>
       </c>
       <c r="B4" t="str">
-        <v>Gunakan format YYYY-MM-DD, contoh 2015-05-14.</v>
+        <v>Isi L (laki-laki) atau P (perempuan).</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Rombel</v>
+        <v>Tanggal Lahir</v>
       </c>
       <c r="B5" t="str">
-        <v>Isi nama rombel persis seperti di menu Data Rombel, contoh 1A. Boleh dikosongkan.</v>
+        <v>Format YYYY-MM-DD, contoh 2015-05-14.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Agama</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Contoh: Islam, Kristen, Katolik, Hindu, Buddha, Konghucu.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Status Keluarga</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Contoh: Anak Kandung, Anak Angkat, Anak Tiri.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Anak Ke</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Angka urutan anak dalam keluarga.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Nama Ayah / Ibu / Wali</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Isi terpisah agar identitas rapor otomatis lengkap.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Pekerjaan Ayah / Ibu / Wali</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Contoh: Petani, Wiraswasta, Ibu Rumah Tangga, PNS.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Rombel</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Nama rombel yang sudah ada, contoh 7A. Boleh dikosongkan.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>Catatan</v>
       </c>
-      <c r="B6" t="str">
-        <v>Hapus baris contoh pada sheet Data Siswa sebelum mengimpor data sebenarnya.</v>
+      <c r="B12" t="str">
+        <v>Baris contoh di bawah boleh dihapus sebelum diunggah.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
bot CS: scope absensi & nilai ke jadwal mengajar HARI INI; RFID + device API; impor RFID; fix nama terwrap
- wa-cs-bot: pengajaranGuruHariIni() — guru 'absensi'/'nilai' hanya menampilkan
  kelas/mapel yang dijadwalkan pada tanggal itu (sesuai jadwal mengajar/mapel).
- RFID: kolom siswa.rfid_uid; /api/absensi-siswa/rfid-scan; pemetaan UID
  (/api/siswa/rfid GET, PUT /api/siswa/:id/rfid); kolom 'RFID UID' di impor Excel
  + template; halaman admin 'Kartu RFID'; mode RFID di halaman scan guru.
- Device API: POST /api/external/v1/absensi/scan (x-api-key, izin absensi:write)
  menerima token QR ATAU rfid_uid — untuk alat mandiri (ESP32/gate).
- Firmware: firmware/esp32-rfid-attendance (sketch + README wiring RC522).
- UI: sel nama siswa whitespace-nowrap (RaporRoster, RekapAbsensi, AbsensiSiswa)
  agar nama tidak terwrap di mobile/tablet.
- tests: wa-cs-bot (day-scope), rfid-device (5), template siswa +RFID UID.
</commit_message>
<xml_diff>
--- a/public/templates/template-import-siswa.xlsx
+++ b/public/templates/template-import-siswa.xlsx
@@ -4,7 +4,6 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Data Siswa" sheetId="1" r:id="rId1"/>
-    <sheet name="Petunjuk" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -398,31 +397,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:X2"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
     <col min="7" max="7" width="16.83203125" customWidth="1"/>
     <col min="8" max="8" width="17.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" customWidth="1"/>
+    <col min="11" max="11" width="15.83203125" customWidth="1"/>
     <col min="12" max="12" width="19.83203125" customWidth="1"/>
-    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="15.83203125" customWidth="1"/>
     <col min="14" max="14" width="16.83203125" customWidth="1"/>
-    <col min="15" max="15" width="16.83203125" customWidth="1"/>
-    <col min="16" max="16" width="16.83203125" customWidth="1"/>
+    <col min="15" max="15" width="15.83203125" customWidth="1"/>
+    <col min="16" max="16" width="15.83203125" customWidth="1"/>
     <col min="17" max="17" width="18.83203125" customWidth="1"/>
-    <col min="18" max="18" width="16.83203125" customWidth="1"/>
+    <col min="18" max="18" width="15.83203125" customWidth="1"/>
     <col min="19" max="19" width="17.83203125" customWidth="1"/>
-    <col min="20" max="20" width="16.83203125" customWidth="1"/>
-    <col min="21" max="21" width="16.83203125" customWidth="1"/>
+    <col min="20" max="20" width="15.83203125" customWidth="1"/>
+    <col min="21" max="21" width="15.83203125" customWidth="1"/>
     <col min="22" max="22" width="18.83203125" customWidth="1"/>
-    <col min="23" max="23" width="16.83203125" customWidth="1"/>
+    <col min="23" max="23" width="15.83203125" customWidth="1"/>
+    <col min="24" max="24" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -495,6 +495,9 @@
       <c r="W1" t="str">
         <v>Rombel</v>
       </c>
+      <c r="X1" t="str">
+        <v>RFID UID</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -533,7 +536,7 @@
       <c r="L2" t="str">
         <v>Anak Kandung</v>
       </c>
-      <c r="M2">
+      <c r="M2" t="str">
         <v>1</v>
       </c>
       <c r="N2" t="str">
@@ -565,111 +568,14 @@
       </c>
       <c r="W2" t="str">
         <v>7A</v>
+      </c>
+      <c r="X2" t="str">
+        <v>04A2B1C3</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B12"/>
-  <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="74.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>PETUNJUK PENGISIAN</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Kolom wajib</v>
-      </c>
-      <c r="B3" t="str">
-        <v>NIS, Nama, dan JK. NIK jika diisi harus tepat 16 digit angka.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>JK</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Isi L (laki-laki) atau P (perempuan).</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Tanggal Lahir</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Format YYYY-MM-DD, contoh 2015-05-14.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Agama</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Contoh: Islam, Kristen, Katolik, Hindu, Buddha, Konghucu.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Status Keluarga</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Contoh: Anak Kandung, Anak Angkat, Anak Tiri.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Anak Ke</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Angka urutan anak dalam keluarga.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Nama Ayah / Ibu / Wali</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Isi terpisah agar identitas rapor otomatis lengkap.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Pekerjaan Ayah / Ibu / Wali</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Contoh: Petani, Wiraswasta, Ibu Rumah Tangga, PNS.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Rombel</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Nama rombel yang sudah ada, contoh 7A. Boleh dikosongkan.</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Catatan</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Baris contoh di bawah boleh dihapus sebelum diunggah.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>